<commit_message>
chore(13-14): remove lga_id from the Public Core form (AC7 — Ministry nod)
The public wizard collects LGA natively (Step 2 → respondents.lgaId), so the form's
lga_id question was a duplicate (wizard UUID vs form slug → dedup fails → asked twice).
Removed survey row 20 from oslsr-public-core-v1.xlsx. Verified: lga_id absent, groups
balanced 6/6, identity block intact, lga_list choices left (unused, harmless). No data
loss. Remaining Task-1/2 (publish both + pin the Core) is operator via the BMAD flow.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/launch-campaign/oslsr-public-core-v1.xlsx
+++ b/docs/launch-campaign/oslsr-public-core-v1.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="399">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="396">
   <si>
     <t>type</t>
   </si>
@@ -193,15 +193,6 @@
   </si>
   <si>
     <t>NIN must be exactly 11 digits</t>
-  </si>
-  <si>
-    <t>select_one lga_list</t>
-  </si>
-  <si>
-    <t>lga_id</t>
-  </si>
-  <si>
-    <t>Local Government Area (LGA)</t>
   </si>
   <si>
     <t>grp_labor</t>
@@ -1586,7 +1577,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -2070,16 +2061,16 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>31</v>
       </c>
       <c r="B20" t="s">
-        <v>61</v>
+        <v>10</v>
       </c>
       <c r="C20" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="D20" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -2096,19 +2087,19 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="C21" t="s">
-        <v>10</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="F21" t="s">
         <v>10</v>
@@ -2122,7 +2113,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
         <v>63</v>
@@ -2131,7 +2122,7 @@
         <v>64</v>
       </c>
       <c r="D22" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E22" t="s">
         <v>65</v>
@@ -2148,19 +2139,19 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C23" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D23" t="s">
         <v>30</v>
       </c>
       <c r="E23" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F23" t="s">
         <v>10</v>
@@ -2186,7 +2177,7 @@
         <v>30</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="F24" t="s">
         <v>10</v>
@@ -2200,19 +2191,19 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>10</v>
       </c>
       <c r="C25" t="s">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E25" t="s">
-        <v>68</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
         <v>10</v>
@@ -2226,19 +2217,19 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>74</v>
       </c>
       <c r="F26" t="s">
         <v>10</v>
@@ -2252,7 +2243,7 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B27" t="s">
         <v>75</v>
@@ -2264,7 +2255,7 @@
         <v>10</v>
       </c>
       <c r="E27" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s">
         <v>10</v>
@@ -2278,16 +2269,16 @@
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="B28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" t="s">
         <v>78</v>
       </c>
-      <c r="C28" t="s">
-        <v>79</v>
-      </c>
       <c r="D28" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E28" t="s">
         <v>10</v>
@@ -2304,7 +2295,7 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="B29" t="s">
         <v>80</v>
@@ -2330,13 +2321,13 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" t="s">
         <v>82</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>83</v>
-      </c>
-      <c r="C30" t="s">
-        <v>84</v>
       </c>
       <c r="D30" t="s">
         <v>30</v>
@@ -2348,21 +2339,21 @@
         <v>10</v>
       </c>
       <c r="G30" t="s">
-        <v>10</v>
+        <v>52</v>
       </c>
       <c r="H30" t="s">
-        <v>10</v>
+        <v>53</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="B31" t="s">
+        <v>84</v>
+      </c>
+      <c r="C31" t="s">
         <v>85</v>
-      </c>
-      <c r="C31" t="s">
-        <v>86</v>
       </c>
       <c r="D31" t="s">
         <v>30</v>
@@ -2374,10 +2365,10 @@
         <v>10</v>
       </c>
       <c r="G31" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="H31" t="s">
-        <v>53</v>
+        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -2385,10 +2376,10 @@
         <v>27</v>
       </c>
       <c r="B32" t="s">
+        <v>86</v>
+      </c>
+      <c r="C32" t="s">
         <v>87</v>
-      </c>
-      <c r="C32" t="s">
-        <v>88</v>
       </c>
       <c r="D32" t="s">
         <v>30</v>
@@ -2408,65 +2399,65 @@
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="B33" t="s">
+        <v>88</v>
+      </c>
+      <c r="C33" t="s">
         <v>89</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>90</v>
       </c>
-      <c r="D33" t="s">
-        <v>30</v>
-      </c>
       <c r="E33" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="F33" t="s">
         <v>10</v>
       </c>
       <c r="G33" t="s">
-        <v>10</v>
+        <v>92</v>
       </c>
       <c r="H33" t="s">
-        <v>10</v>
+        <v>93</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B34" t="s">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="C34" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="E34" t="s">
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="F34" t="s">
         <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="H34" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B35" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="C35" t="s">
-        <v>10</v>
+        <v>95</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
@@ -2486,7 +2477,7 @@
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="B36" t="s">
         <v>97</v>
@@ -2495,7 +2486,7 @@
         <v>98</v>
       </c>
       <c r="D36" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E36" t="s">
         <v>10</v>
@@ -2512,16 +2503,16 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
         <v>99</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>100</v>
       </c>
-      <c r="C37" t="s">
-        <v>101</v>
-      </c>
       <c r="D37" t="s">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s">
         <v>10</v>
@@ -2530,24 +2521,24 @@
         <v>10</v>
       </c>
       <c r="G37" t="s">
-        <v>10</v>
+        <v>92</v>
       </c>
       <c r="H37" t="s">
-        <v>10</v>
+        <v>93</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="B38" t="s">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="C38" t="s">
-        <v>103</v>
+        <v>10</v>
       </c>
       <c r="D38" t="s">
-        <v>93</v>
+        <v>10</v>
       </c>
       <c r="E38" t="s">
         <v>10</v>
@@ -2556,21 +2547,21 @@
         <v>10</v>
       </c>
       <c r="G38" t="s">
-        <v>95</v>
+        <v>10</v>
       </c>
       <c r="H38" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="B39" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="C39" t="s">
-        <v>10</v>
+        <v>102</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -2590,13 +2581,13 @@
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B40" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" t="s">
         <v>104</v>
-      </c>
-      <c r="C40" t="s">
-        <v>105</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
@@ -2616,16 +2607,16 @@
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B41" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" t="s">
         <v>106</v>
       </c>
-      <c r="C41" t="s">
-        <v>107</v>
-      </c>
       <c r="D41" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="E41" t="s">
         <v>10</v>
@@ -2645,16 +2636,16 @@
         <v>27</v>
       </c>
       <c r="B42" t="s">
+        <v>107</v>
+      </c>
+      <c r="C42" t="s">
         <v>108</v>
-      </c>
-      <c r="C42" t="s">
-        <v>109</v>
       </c>
       <c r="D42" t="s">
         <v>30</v>
       </c>
       <c r="E42" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="F42" t="s">
         <v>10</v>
@@ -2668,19 +2659,19 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B43" t="s">
-        <v>110</v>
+        <v>10</v>
       </c>
       <c r="C43" t="s">
-        <v>111</v>
+        <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E43" t="s">
-        <v>112</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
         <v>10</v>
@@ -2689,38 +2680,12 @@
         <v>10</v>
       </c>
       <c r="H43" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>31</v>
-      </c>
-      <c r="B44" t="s">
-        <v>10</v>
-      </c>
-      <c r="C44" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" t="s">
-        <v>10</v>
-      </c>
-      <c r="F44" t="s">
-        <v>10</v>
-      </c>
-      <c r="G44" t="s">
-        <v>10</v>
-      </c>
-      <c r="H44" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2731,7 +2696,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -2742,1492 +2707,1492 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B2" t="s">
         <v>30</v>
       </c>
       <c r="C2" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B5" t="s">
         <v>117</v>
       </c>
-      <c r="B5" t="s">
-        <v>120</v>
-      </c>
       <c r="C5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C6" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C7" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>121</v>
+      </c>
+      <c r="B8" t="s">
         <v>124</v>
       </c>
-      <c r="B8" t="s">
-        <v>127</v>
-      </c>
       <c r="C8" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C9" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B10" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C10" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C11" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C12" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>132</v>
+      </c>
+      <c r="B13" t="s">
         <v>135</v>
       </c>
-      <c r="B13" t="s">
-        <v>138</v>
-      </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B14" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C14" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B15" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C15" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B16" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C16" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C17" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B18" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C18" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B19" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C19" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C20" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B21" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C21" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" t="s">
         <v>154</v>
       </c>
-      <c r="B22" t="s">
-        <v>157</v>
-      </c>
       <c r="C22" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B23" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C23" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B24" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C24" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B25" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C25" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B26" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C26" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B27" t="s">
         <v>164</v>
       </c>
-      <c r="B27" t="s">
-        <v>167</v>
-      </c>
       <c r="C27" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B28" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C28" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C29" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B30" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C30" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B31" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C31" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B32" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C32" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
+        <v>174</v>
+      </c>
+      <c r="B33" t="s">
         <v>177</v>
       </c>
-      <c r="B33" t="s">
-        <v>180</v>
-      </c>
       <c r="C33" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B34" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C34" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B35" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C35" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B36" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C36" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B37" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C37" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
+        <v>185</v>
+      </c>
+      <c r="B38" t="s">
         <v>188</v>
       </c>
-      <c r="B38" t="s">
-        <v>191</v>
-      </c>
       <c r="C38" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B39" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C39" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B40" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C40" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>192</v>
+      </c>
+      <c r="B41" t="s">
         <v>195</v>
       </c>
-      <c r="B41" t="s">
-        <v>198</v>
-      </c>
       <c r="C41" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B42" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C42" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B43" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C43" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B44" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C44" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B45" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C45" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B46" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C46" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B47" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C47" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B48" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C48" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B49" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C49" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B50" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C50" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B51" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C51" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B52" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C52" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B53" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C53" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B54" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C54" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B55" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C55" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B56" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C56" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B57" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C57" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B58" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C58" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B59" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="C59" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B60" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C60" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B61" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C61" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B62" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C62" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B63" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C63" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B64" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="C64" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B65" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C65" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
     </row>
     <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B66" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C66" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B67" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="C67" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B68" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="C68" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B69" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C69" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B70" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="C70" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B71" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="C71" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B72" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C72" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B73" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C73" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>259</v>
+      </c>
+      <c r="B74" t="s">
         <v>262</v>
       </c>
-      <c r="B74" t="s">
-        <v>265</v>
-      </c>
       <c r="C74" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B75" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="C75" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B76" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C76" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B77" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="C77" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B78" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="C78" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B79" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C79" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B80" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C80" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B81" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C81" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B82" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C82" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B83" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="C83" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B84" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="C84" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B85" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C85" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B86" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="C86" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B87" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C87" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B88" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="C88" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B89" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C89" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B90" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="C90" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B91" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C91" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B92" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="C92" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B93" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C93" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B94" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C94" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B95" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C95" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B96" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C96" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B97" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C97" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B98" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C98" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
     </row>
     <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B99" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C99" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B100" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="C100" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B101" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="C101" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B102" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="C102" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B103" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="C103" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B104" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="C104" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B105" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="C105" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B106" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="C106" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B107" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="C107" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B108" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C108" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B109" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="C109" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B110" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="C110" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B111" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="C111" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B112" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="C112" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B113" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="C113" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B114" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="C114" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B115" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="C115" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B116" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="C116" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B117" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="C117" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B118" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C118" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B119" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="C119" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B120" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C120" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B121" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="C121" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B122" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C122" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B123" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="C123" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B124" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C124" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B125" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C125" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B126" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="C126" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B127" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C127" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B128" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C128" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B129" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C129" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B130" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C130" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B131" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C131" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B132" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="C132" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="B133" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="C133" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B134" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C134" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
+        <v>382</v>
+      </c>
+      <c r="B135" t="s">
         <v>385</v>
       </c>
-      <c r="B135" t="s">
-        <v>388</v>
-      </c>
       <c r="C135" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="B136" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C136" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -4238,34 +4203,34 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>388</v>
+      </c>
+      <c r="B1" t="s">
+        <v>389</v>
+      </c>
+      <c r="C1" t="s">
+        <v>390</v>
+      </c>
+      <c r="D1" t="s">
         <v>391</v>
-      </c>
-      <c r="B1" t="s">
-        <v>392</v>
-      </c>
-      <c r="C1" t="s">
-        <v>393</v>
-      </c>
-      <c r="D1" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>392</v>
+      </c>
+      <c r="B2" t="s">
+        <v>393</v>
+      </c>
+      <c r="C2" t="s">
+        <v>394</v>
+      </c>
+      <c r="D2" t="s">
         <v>395</v>
-      </c>
-      <c r="B2" t="s">
-        <v>396</v>
-      </c>
-      <c r="C2" t="s">
-        <v>397</v>
-      </c>
-      <c r="D2" t="s">
-        <v>398</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>